<commit_message>
v6.0 特性扩展：M10/M12/M22/M24/M26/M30/M36 新增特性 + 更新人物MD + 重新生成Excel
</commit_message>
<xml_diff>
--- a/boss_traits_v6.xlsx
+++ b/boss_traits_v6.xlsx
@@ -719,16 +719,16 @@
         <v>3</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>护体</t>
+          <t>护体(旧)、破防贯通</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
-          <t>开场护体盾30%HP，高防稳守</t>
+          <t>开场护体盾30%HP；玩家DEF剩50%</t>
         </is>
       </c>
     </row>
@@ -752,16 +752,16 @@
         <v>5</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>破防贯通、断筋</t>
+          <t>破防贯通、断筋、护体真气、低血狂暴</t>
         </is>
       </c>
       <c r="G6" s="9" t="inlineStr">
         <is>
-          <t>破防贯通（玩家DEF×50%）；每回合断筋+5，上限15层</t>
+          <t>破防+断筋+护体30%；≤30%HP ATK×1.5, SPD×1.5</t>
         </is>
       </c>
     </row>
@@ -917,16 +917,16 @@
         <v>4</v>
       </c>
       <c r="E11" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F11" s="11" t="inlineStr">
         <is>
-          <t>血刃、断脉</t>
+          <t>血刃、断脉、影步</t>
         </is>
       </c>
       <c r="G11" s="11" t="inlineStr">
         <is>
-          <t>每回合流血+4（血刃）、断脉+4，上限15层</t>
+          <t>每回合流血+4、断脉+4；基础闪避75%，≤50%HP闪避×1.5</t>
         </is>
       </c>
     </row>
@@ -950,16 +950,16 @@
         <v>7</v>
       </c>
       <c r="E12" s="12" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F12" s="13" t="inlineStr">
         <is>
-          <t>天罡护体、低血狂暴</t>
+          <t>天罡护体、低血狂暴、血刃、寒气逼人</t>
         </is>
       </c>
       <c r="G12" s="13" t="inlineStr">
         <is>
-          <t>开场30%HP天罡护体；≤30%HP ATK×1.5，SPEED×2.1，持续5回合</t>
+          <t>开场30%护体；≤30%HP狂暴；每回合流血+5、寒气+5</t>
         </is>
       </c>
     </row>
@@ -983,16 +983,16 @@
         <v>5</v>
       </c>
       <c r="E13" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F13" s="9" t="inlineStr">
         <is>
-          <t>断筋</t>
+          <t>断筋、低血狂暴</t>
         </is>
       </c>
       <c r="G13" s="9" t="inlineStr">
         <is>
-          <t>每回合断筋+5，上限15层</t>
+          <t>每回合断筋+5；≤30%HP ATK×1.5, SPD×1.5</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
       </c>
       <c r="G14" s="9" t="inlineStr">
         <is>
-          <t>≤50%HP天罡净化+回血30%；≤30%HP ATK×1.5，SPEED×1.5，持续5回合</t>
+          <t>≤50%HP天罡净化+回血30%；≤30%HP狂暴</t>
         </is>
       </c>
     </row>
@@ -1049,16 +1049,16 @@
         <v>6</v>
       </c>
       <c r="E15" s="14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F15" s="15" t="inlineStr">
         <is>
-          <t>天罡护体</t>
+          <t>天罡护体、破防贯通</t>
         </is>
       </c>
       <c r="G15" s="15" t="inlineStr">
         <is>
-          <t>开场30%HP天罡护体</t>
+          <t>开场30%护体；玩家DEF剩50%，每次命中DEF-5%</t>
         </is>
       </c>
     </row>
@@ -1091,7 +1091,7 @@
       </c>
       <c r="G16" s="15" t="inlineStr">
         <is>
-          <t>开场30%HP天罡护体；每回合流血+6（血刃），上限15层</t>
+          <t>开场30%护体；每回合流血+6（血刃），上限15层</t>
         </is>
       </c>
     </row>
@@ -1124,7 +1124,7 @@
       </c>
       <c r="G17" s="15" t="inlineStr">
         <is>
-          <t>≤50%HP天罡净化+回血30%；每回合断脉+6、断筋+6，上限15层</t>
+          <t>≤50%HP净化+回血30%；每回合断脉+6、断筋+6</t>
         </is>
       </c>
     </row>
@@ -1148,16 +1148,16 @@
         <v>10</v>
       </c>
       <c r="E18" s="16" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F18" s="17" t="inlineStr">
         <is>
-          <t>断脉、断筋</t>
+          <t>断脉、断筋、天罡护体、天罡净化、天罡燃命</t>
         </is>
       </c>
       <c r="G18" s="17" t="inlineStr">
         <is>
-          <t>每回合断脉+10、断筋+10，上限15层</t>
+          <t>每回合断脉+10、断筋+10；开场30%护体；≤50%净化；≤10%燃命</t>
         </is>
       </c>
     </row>
@@ -1261,7 +1261,7 @@
       </c>
       <c r="C5" s="18" t="inlineStr">
         <is>
-          <t>每回合寒气+n，上限15层（每层减内力2%、减速2%）</t>
+          <t>每回合寒气+n，上限25层（每层减内力2%、减速2%）</t>
         </is>
       </c>
     </row>
@@ -1312,7 +1312,7 @@
       </c>
       <c r="C8" s="18" t="inlineStr">
         <is>
-          <t>≤30%HP ATK×1.5, SPEED×n×0.3，持续5回合</t>
+          <t>≤30%HP ATK×1.5, SPD×n×0.3，持续5回合</t>
         </is>
       </c>
     </row>
@@ -1397,7 +1397,7 @@
       </c>
       <c r="C13" s="18" t="inlineStr">
         <is>
-          <t>≤10%HP自动释放，ATK×2,SPEED×2,DEF×0.5，持续5回合</t>
+          <t>≤10%HP自动释放，ATK×2, SPD×2, DEF×0.5，持续5回合</t>
         </is>
       </c>
     </row>
@@ -1409,7 +1409,7 @@
       </c>
       <c r="B14" s="18" t="inlineStr">
         <is>
-          <t>护体</t>
+          <t>护体(旧)</t>
         </is>
       </c>
       <c r="C14" s="18" t="inlineStr">
@@ -1432,26 +1432,26 @@
   <dimension ref="A1:N18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Boss / 阶级</t>
+          <t>Boss / 特性</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -1516,7 +1516,7 @@
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>护体</t>
+          <t>护体(旧)</t>
         </is>
       </c>
     </row>
@@ -1602,7 +1602,11 @@
           <t>M10 护法副将·杨震 [3阶]</t>
         </is>
       </c>
-      <c r="B5" s="19" t="inlineStr"/>
+      <c r="B5" s="20" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="C5" s="19" t="inlineStr"/>
       <c r="D5" s="19" t="inlineStr"/>
       <c r="E5" s="19" t="inlineStr"/>
@@ -1640,9 +1644,17 @@
       <c r="E6" s="19" t="inlineStr"/>
       <c r="F6" s="19" t="inlineStr"/>
       <c r="G6" s="19" t="inlineStr"/>
-      <c r="H6" s="19" t="inlineStr"/>
+      <c r="H6" s="20" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="I6" s="19" t="inlineStr"/>
-      <c r="J6" s="19" t="inlineStr"/>
+      <c r="J6" s="20" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="K6" s="19" t="inlineStr"/>
       <c r="L6" s="19" t="inlineStr"/>
       <c r="M6" s="19" t="inlineStr"/>
@@ -1773,7 +1785,11 @@
       </c>
       <c r="G11" s="19" t="inlineStr"/>
       <c r="H11" s="19" t="inlineStr"/>
-      <c r="I11" s="19" t="inlineStr"/>
+      <c r="I11" s="20" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="J11" s="19" t="inlineStr"/>
       <c r="K11" s="19" t="inlineStr"/>
       <c r="L11" s="19" t="inlineStr"/>
@@ -1789,8 +1805,16 @@
       <c r="B12" s="19" t="inlineStr"/>
       <c r="C12" s="19" t="inlineStr"/>
       <c r="D12" s="19" t="inlineStr"/>
-      <c r="E12" s="19" t="inlineStr"/>
-      <c r="F12" s="19" t="inlineStr"/>
+      <c r="E12" s="20" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F12" s="20" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="G12" s="19" t="inlineStr"/>
       <c r="H12" s="20" t="inlineStr">
         <is>
@@ -1824,7 +1848,11 @@
       <c r="E13" s="19" t="inlineStr"/>
       <c r="F13" s="19" t="inlineStr"/>
       <c r="G13" s="19" t="inlineStr"/>
-      <c r="H13" s="19" t="inlineStr"/>
+      <c r="H13" s="20" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="I13" s="19" t="inlineStr"/>
       <c r="J13" s="19" t="inlineStr"/>
       <c r="K13" s="19" t="inlineStr"/>
@@ -1866,7 +1894,11 @@
           <t>M30 烽火统领·霍烽 [6阶]</t>
         </is>
       </c>
-      <c r="B15" s="19" t="inlineStr"/>
+      <c r="B15" s="20" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="C15" s="19" t="inlineStr"/>
       <c r="D15" s="19" t="inlineStr"/>
       <c r="E15" s="19" t="inlineStr"/>
@@ -1967,9 +1999,21 @@
       <c r="H18" s="19" t="inlineStr"/>
       <c r="I18" s="19" t="inlineStr"/>
       <c r="J18" s="19" t="inlineStr"/>
-      <c r="K18" s="19" t="inlineStr"/>
-      <c r="L18" s="19" t="inlineStr"/>
-      <c r="M18" s="19" t="inlineStr"/>
+      <c r="K18" s="20" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="L18" s="20" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="M18" s="20" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="N18" s="19" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>